<commit_message>
Update data from docs CSVs (no duplicates), Last Updated 16th May 2026
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Pie Chart Data.XLSX
+++ b/docs/Pie Chart Data.XLSX
@@ -1,31 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Portfolio\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C321F542-3366-452C-B5CE-BAC62AC4A3E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E0436C9-2C72-4158-88D3-D45134527D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="12216" windowHeight="18816" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>AI Hyperscalers Stocks</t>
   </si>
@@ -42,16 +53,37 @@
     <t>Japanese Stocks</t>
   </si>
   <si>
-    <t>Gold ETF</t>
-  </si>
-  <si>
     <t>Healthcare Stocks</t>
   </si>
   <si>
     <t>SaaS Stocks</t>
   </si>
   <si>
-    <t>Semiconductor Stocks</t>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>#8D9196</t>
+  </si>
+  <si>
+    <t>#7BD1DD</t>
+  </si>
+  <si>
+    <t>#F99E3F</t>
+  </si>
+  <si>
+    <t>#FF3030</t>
+  </si>
+  <si>
+    <t>#F5E162</t>
+  </si>
+  <si>
+    <t>#F184D7</t>
+  </si>
+  <si>
+    <t>#62B9D1</t>
+  </si>
+  <si>
+    <t>Gold ETF (GLDM)</t>
   </si>
 </sst>
 </file>
@@ -371,77 +403,99 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="2">
-        <v>0.252</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.28100000000000003</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="1">
-        <v>0.24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.19900000000000001</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>0.16300000000000001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.214</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="2">
-        <v>0.113</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>9.8000000000000004E-2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="2">
+        <v>6.7000000000000004E-2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="2">
-        <v>6.2E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B7" s="2">
+        <v>0.09</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="2">
-        <v>7.8E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
       <c r="B8" s="2">
-        <v>5.2999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2">
-        <v>2.5999999999999999E-2</v>
-      </c>
+        <v>5.0999999999999997E-2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B9" s="2"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B11" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>